<commit_message>
Bài 31 - DataProvider
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/crm_data.xlsx
+++ b/src/test/resources/testdata/crm_data.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ANHTESTER\SeleniumJava\Course_SeleniumJava_012026\SeleniumTestNGParallel012026\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48672D3A-FCE1-4547-92A6-5E4DB804881A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8EEE61-F589-4C73-8E76-74B1DE273084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4872" yWindow="1848" windowWidth="22704" windowHeight="13872" xr2:uid="{4FDC73F2-BBBB-4648-B85A-668934903B71}"/>
+    <workbookView xWindow="5220" yWindow="2196" windowWidth="22704" windowHeight="13872" xr2:uid="{4FDC73F2-BBBB-4648-B85A-668934903B71}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="AddCustomer" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Login!$A$1:$D$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
     <t>EMAIL</t>
   </si>
@@ -99,13 +100,90 @@
   </si>
   <si>
     <t>SELENIUM JAVA</t>
+  </si>
+  <si>
+    <t>COMPANY</t>
+  </si>
+  <si>
+    <t>VAT</t>
+  </si>
+  <si>
+    <t>ADDRESS</t>
+  </si>
+  <si>
+    <t>PHONE</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>Microsoft</t>
+  </si>
+  <si>
+    <t>NVIDIA</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>FPT</t>
+  </si>
+  <si>
+    <t>VN</t>
+  </si>
+  <si>
+    <t>CHINA</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t>1234</t>
+  </si>
+  <si>
+    <t>1234567</t>
+  </si>
+  <si>
+    <t>SAMSUNG</t>
+  </si>
+  <si>
+    <t>VIETTEL</t>
+  </si>
+  <si>
+    <t>VNPT</t>
+  </si>
+  <si>
+    <t>KOREA</t>
+  </si>
+  <si>
+    <t>0986875</t>
+  </si>
+  <si>
+    <t>099864745</t>
+  </si>
+  <si>
+    <t>077547935</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
@@ -133,19 +211,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="9"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="9"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -159,27 +237,23 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="none">
-        <fgColor rgb="4CAF50"/>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4CAF50"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="4CAF50"/>
+        <fgColor rgb="FFE53935"/>
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="none">
-        <fgColor rgb="E53935"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="E53935"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
-    </fill>
-    <fill>
-      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -195,7 +269,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -210,13 +284,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyAlignment="true" applyFill="true" applyFont="true">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyAlignment="true" applyFill="true" applyFont="true">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyAlignment="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -557,10 +637,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="22.53515625"/>
-    <col min="2" max="2" customWidth="true" width="17.15234375"/>
-    <col min="3" max="3" customWidth="true" style="4" width="35.53515625"/>
-    <col min="4" max="4" customWidth="true" width="18.921875"/>
+    <col min="1" max="1" width="22.53515625" customWidth="1"/>
+    <col min="2" max="2" width="17.15234375" customWidth="1"/>
+    <col min="3" max="3" width="35.53515625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -587,7 +667,7 @@
       <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s" s="6">
+      <c r="D2" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -601,7 +681,7 @@
       <c r="C3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s" s="7">
+      <c r="D3" s="7" t="s">
         <v>17</v>
       </c>
     </row>
@@ -615,7 +695,7 @@
       <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s" s="8">
+      <c r="D4" s="8" t="s">
         <v>18</v>
       </c>
     </row>
@@ -674,4 +754,134 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId7"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B588024-5EE6-43D3-A77D-642D8CA04BE6}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.61328125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="9.23046875" style="4"/>
+    <col min="3" max="3" width="13.23046875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.3046875" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="9.23046875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="4">
+        <v>20</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="4">
+        <v>25.5</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="4">
+        <v>30.7</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>